<commit_message>
fix: Local Sbase 를 MVA 로 (뿌리 = 변환기)
엔진은 AC_gen_local_S / (S_base/1e6) 로 쓴다 — 이 칸은 MVA 다.
그런데 unigrid_convert.py 가 MATPOWER mBase · PSS/E MBASE 에 1e6 을
곱해 VA 로 써 왔다. droop 계수가 100만 배 어긋난다.

  src/unigrid_convert.py  MATPOWER 경로 122행 · PSS/E 경로 357행

이미 만들어진 케이스 4개도 같이 바로잡았다 (그 열만 1e6 으로 나눔):
  AConly_case14 5줄 · AConly_case118 54줄 ·
  AConly_case118_psse 54줄 · AConly_psse_3W_unigrid_easy 7줄

확인
  - 고친 변환기로 case14.m 를 다시 읽으니 Local Sbase = 100 (mBase 그대로)
  - 케이스 4개 결과 전부 그대로 (그 넷엔 droop 발전기가 없어 잠복해 있었다)
  - 회귀 11건 같음 · scenario 테스트 통과
  - 정말 문제였나: 71bus(발전기 4대 전부 droop) 의 Local Sbase 를 100만 배
    하니 주파수 49.676 → 50.000 Hz, 전압최저 0.9764 → 0.9670 으로 어긋남

DC 발전기 Local Sbase 는 전 케이스 정상 (1 · 25 · 0.001).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cases/AConly_case118.xlsx
+++ b/cases/AConly_case118.xlsx
@@ -15126,7 +15126,7 @@
         <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K2" t="n">
         <v>1e-06</v>
@@ -15161,7 +15161,7 @@
         <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K3" t="n">
         <v>1e-06</v>
@@ -15196,7 +15196,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K4" t="n">
         <v>1e-06</v>
@@ -15231,7 +15231,7 @@
         <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K5" t="n">
         <v>1e-06</v>
@@ -15266,7 +15266,7 @@
         <v>1</v>
       </c>
       <c r="J6" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K6" t="n">
         <v>1e-06</v>
@@ -15301,7 +15301,7 @@
         <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K7" t="n">
         <v>1e-06</v>
@@ -15336,7 +15336,7 @@
         <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K8" t="n">
         <v>1e-06</v>
@@ -15371,7 +15371,7 @@
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K9" t="n">
         <v>1e-06</v>
@@ -15406,7 +15406,7 @@
         <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K10" t="n">
         <v>1e-06</v>
@@ -15441,7 +15441,7 @@
         <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K11" t="n">
         <v>1e-06</v>
@@ -15476,7 +15476,7 @@
         <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K12" t="n">
         <v>1e-06</v>
@@ -15511,7 +15511,7 @@
         <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K13" t="n">
         <v>1e-06</v>
@@ -15546,7 +15546,7 @@
         <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K14" t="n">
         <v>1e-06</v>
@@ -15581,7 +15581,7 @@
         <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K15" t="n">
         <v>1e-06</v>
@@ -15616,7 +15616,7 @@
         <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K16" t="n">
         <v>1e-06</v>
@@ -15651,7 +15651,7 @@
         <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K17" t="n">
         <v>1e-06</v>
@@ -15686,7 +15686,7 @@
         <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K18" t="n">
         <v>1e-06</v>
@@ -15721,7 +15721,7 @@
         <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K19" t="n">
         <v>1e-06</v>
@@ -15756,7 +15756,7 @@
         <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K20" t="n">
         <v>1e-06</v>
@@ -15791,7 +15791,7 @@
         <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K21" t="n">
         <v>1e-06</v>
@@ -15826,7 +15826,7 @@
         <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K22" t="n">
         <v>1e-06</v>
@@ -15861,7 +15861,7 @@
         <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K23" t="n">
         <v>1e-06</v>
@@ -15896,7 +15896,7 @@
         <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K24" t="n">
         <v>1e-06</v>
@@ -15931,7 +15931,7 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K25" t="n">
         <v>1e-06</v>
@@ -15966,7 +15966,7 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K26" t="n">
         <v>1e-06</v>
@@ -16001,7 +16001,7 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K27" t="n">
         <v>1e-06</v>
@@ -16036,7 +16036,7 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K28" t="n">
         <v>1e-06</v>
@@ -16071,7 +16071,7 @@
         <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K29" t="n">
         <v>1e-06</v>
@@ -16106,7 +16106,7 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K30" t="n">
         <v>1e-06</v>
@@ -16141,7 +16141,7 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K31" t="n">
         <v>1e-06</v>
@@ -16176,7 +16176,7 @@
         <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K32" t="n">
         <v>1e-06</v>
@@ -16211,7 +16211,7 @@
         <v>1</v>
       </c>
       <c r="J33" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K33" t="n">
         <v>1e-06</v>
@@ -16246,7 +16246,7 @@
         <v>1</v>
       </c>
       <c r="J34" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K34" t="n">
         <v>1e-06</v>
@@ -16281,7 +16281,7 @@
         <v>1</v>
       </c>
       <c r="J35" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K35" t="n">
         <v>1e-06</v>
@@ -16316,7 +16316,7 @@
         <v>1</v>
       </c>
       <c r="J36" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K36" t="n">
         <v>1e-06</v>
@@ -16351,7 +16351,7 @@
         <v>1</v>
       </c>
       <c r="J37" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K37" t="n">
         <v>1e-06</v>
@@ -16386,7 +16386,7 @@
         <v>1</v>
       </c>
       <c r="J38" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K38" t="n">
         <v>1e-06</v>
@@ -16421,7 +16421,7 @@
         <v>1</v>
       </c>
       <c r="J39" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K39" t="n">
         <v>1e-06</v>
@@ -16456,7 +16456,7 @@
         <v>1</v>
       </c>
       <c r="J40" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K40" t="n">
         <v>1e-06</v>
@@ -16491,7 +16491,7 @@
         <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K41" t="n">
         <v>1e-06</v>
@@ -16526,7 +16526,7 @@
         <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K42" t="n">
         <v>1e-06</v>
@@ -16561,7 +16561,7 @@
         <v>1</v>
       </c>
       <c r="J43" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K43" t="n">
         <v>1e-06</v>
@@ -16596,7 +16596,7 @@
         <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K44" t="n">
         <v>1e-06</v>
@@ -16631,7 +16631,7 @@
         <v>1</v>
       </c>
       <c r="J45" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K45" t="n">
         <v>1e-06</v>
@@ -16666,7 +16666,7 @@
         <v>1</v>
       </c>
       <c r="J46" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K46" t="n">
         <v>1e-06</v>
@@ -16701,7 +16701,7 @@
         <v>1</v>
       </c>
       <c r="J47" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K47" t="n">
         <v>1e-06</v>
@@ -16736,7 +16736,7 @@
         <v>1</v>
       </c>
       <c r="J48" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K48" t="n">
         <v>1e-06</v>
@@ -16771,7 +16771,7 @@
         <v>1</v>
       </c>
       <c r="J49" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K49" t="n">
         <v>1e-06</v>
@@ -16806,7 +16806,7 @@
         <v>1</v>
       </c>
       <c r="J50" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K50" t="n">
         <v>1e-06</v>
@@ -16841,7 +16841,7 @@
         <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K51" t="n">
         <v>1e-06</v>
@@ -16876,7 +16876,7 @@
         <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K52" t="n">
         <v>1e-06</v>
@@ -16911,7 +16911,7 @@
         <v>1</v>
       </c>
       <c r="J53" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K53" t="n">
         <v>1e-06</v>
@@ -16946,7 +16946,7 @@
         <v>1</v>
       </c>
       <c r="J54" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K54" t="n">
         <v>1e-06</v>
@@ -16981,7 +16981,7 @@
         <v>1</v>
       </c>
       <c r="J55" t="n">
-        <v>100000000</v>
+        <v>100</v>
       </c>
       <c r="K55" t="n">
         <v>1e-06</v>

</xml_diff>